<commit_message>
🤖 AI 채점 엔진 자동 배포: 2026-05-16 18:06:59
</commit_message>
<xml_diff>
--- a/storage/글쓰기대회_결과리스트.xlsx
+++ b/storage/글쓰기대회_결과리스트.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M7"/>
+  <dimension ref="A1:M8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -753,6 +753,55 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-05-16 18:06:59</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>학생</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+      <c r="D8" t="n">
+        <v>1500</v>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>이타적인 행동이 만드는 변화라는 멋진 주제로 글을 시작해 주었네요. 특히, 마더 테레사 수녀님처럼 대가 없이 다른 사람들을 도왔던 경험을 떠올리며, "정말로 그는 이타적인 사람이라는 것이 느껴집니다"라고 표현한 부분에서 깊은 공감이 느껴졌습니다. 황무지에 숲을 일군 부피에처럼, 우리 주변의 작은 실천들이 모여 세상을 긍정적으로 바꿀 수 있다는 깨달음을 주었어요. 앞으로도 이타적인 마음으로 따뜻한 변화를 만들어가는 멋진 학생이 되기를 응원합니다.</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>상</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>상</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>하</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>상</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>상</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 AI 채점 엔진 자동 배포: 2026-05-16 18:11:00
</commit_message>
<xml_diff>
--- a/storage/글쓰기대회_결과리스트.xlsx
+++ b/storage/글쓰기대회_결과리스트.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -802,6 +802,55 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-05-16 18:10:59</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>이주아</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr"/>
+      <c r="D9" t="n">
+        <v>1352</v>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>이주아 학생은 '프랑스 혁명 해결하기'와 '우리가 원하는 세상'이라는 제목처럼, 불평등한 사회를 바꾸려는 뜨거운 열망을 담아 글을 써 주었네요. 장발장이 '오직 먹여살리려고' 빵을 훔쳤음에도 억울하게 감옥살이를 했다는 구절에서 불합리한 현실에 대한 공감과 비판 의식이 돋보였습니다. 루소의 사회계약설을 인용하며 자유롭고 평등한 세상을 꿈꾸는 학생의 마음이 잘 느껴졌어요. 앞으로도 주변의 불의에 관심을 가지고 더 나은 사회를 위해 노력하기를 응원합니다.</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>상</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>상</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>상</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>중</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>상</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 AI 채점 엔진 자동 배포: 2026-05-22 11:09:44
</commit_message>
<xml_diff>
--- a/storage/글쓰기대회_결과리스트.xlsx
+++ b/storage/글쓰기대회_결과리스트.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -851,6 +851,55 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-05-22 11:09:44</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>김아인</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="n">
+        <v>1020</v>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>‘혼자서는 못 살아요!’라는 제목처럼, 인간은 사회적 동물이라는 깊은 통찰을 담은 글을 읽었습니다. 로빈슨 크루소가 의식주를 모두 충족했음에도 '함께 지내줄 다른 사람'이 없어 외로움을 느꼈다는 부분에서 인간 본연의 사회성을 정확히 짚어냈습니다. 현대 사회의 '나홀로족'에 대한 분석에서도 '생활 방식만 달라질 뿐 인간들은 서로에게 연결되어 있다'는 따뜻한 시선이 돋보였어요. 앞으로도 주변 사람들과의 소중한 연결고리를 잘 가꾸며 함께 성장해 나가기를 응원합니다.</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>상</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>상</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>하</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>하</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>상</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
🤖 AI 채점 엔진 자동 배포: 2026-05-23 18:01:03
</commit_message>
<xml_diff>
--- a/storage/글쓰기대회_결과리스트.xlsx
+++ b/storage/글쓰기대회_결과리스트.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
+  <dimension ref="A1:M11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -900,6 +900,45 @@
         </is>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-05-23 18:01:01</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>양해원</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr"/>
+      <c r="D11" t="n">
+        <v>1600</v>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>“인생에서 배울 것의 절반”이라는 멋진 제목처럼, 열하일기를 통해 세상을 바라보는 새로운 시선을 얻었네요. 특히 박지원 선생이 ‘기와 조각과 똥 덩어리’에서도 가치를 발견한 일화에서, 겉모습만으로 판단하지 않겠다는 다짐이 인상 깊었습니다. 신분 고하를 막론하고 배움을 권했던 박지원처럼, 앞으로도 편견 없이 세상을 탐구하며 지혜롭게 성장하기를 응원합니다.</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
+        <v>8</v>
+      </c>
+      <c r="J11" t="n">
+        <v>8</v>
+      </c>
+      <c r="K11" t="n">
+        <v>9</v>
+      </c>
+      <c r="L11" t="n">
+        <v>8</v>
+      </c>
+      <c r="M11" t="n">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>